<commit_message>
Fix technical inventory XLSX generator per PR review
- Enforce minimum column width of 10 in autosize
- Add openpyxl to backend requirements and tech stack docs
- Expand schema sheet to all 21 database tables
- Align external APIs sheet with TECHNICAL_INVENTORY.md (17 services)
- Regenerate TECHNICAL_INVENTORY.xlsx

Co-authored-by: Soldier0x0 <Soldier0x0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TECHNICAL_INVENTORY.xlsx
+++ b/TECHNICAL_INVENTORY.xlsx
@@ -418,13 +418,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -644,6 +644,28 @@
       <c r="D10" t="inlineStr">
         <is>
           <t>Client PDF reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Spreadsheet generation</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>openpyxl</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3.1.5</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TECHNICAL_INVENTORY.xlsx script</t>
         </is>
       </c>
     </row>
@@ -658,14 +680,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -741,7 +763,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>NVD description</t>
+          <t>NVD English description</t>
         </is>
       </c>
     </row>
@@ -764,7 +786,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CVSS v3 base</t>
+          <t>CVSS v3 base score</t>
         </is>
       </c>
     </row>
@@ -810,7 +832,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Publish timestamp</t>
+          <t>ISO publish timestamp</t>
         </is>
       </c>
     </row>
@@ -833,7 +855,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Last modified</t>
+          <t>ISO last-modified</t>
         </is>
       </c>
     </row>
@@ -860,7 +882,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>JSON vendor:product</t>
+          <t>JSON array vendor:product</t>
         </is>
       </c>
     </row>
@@ -883,7 +905,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Primary ATT&amp;CK ID</t>
+          <t>Primary ATT&amp;CK ID from refs</t>
         </is>
       </c>
     </row>
@@ -906,7 +928,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Plain-English summary</t>
+          <t>Plain-English summary (KEV/OSV)</t>
         </is>
       </c>
     </row>
@@ -956,7 +978,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>EPSS probability</t>
+          <t>Latest EPSS probability</t>
         </is>
       </c>
     </row>
@@ -983,7 +1005,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Public PoC flag</t>
+          <t>Public PoC/exploit flag</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1032,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Patch ref flag</t>
+          <t>Patch reference detected</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1059,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AI/ML relevance</t>
+          <t>AI/ML relevance flag</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1086,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>JSON URLs</t>
+          <t>JSON reference URLs</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1113,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>JSON CWEs</t>
+          <t>JSON CWE list</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1140,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Row update</t>
+          <t>Row update time</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1167,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>JSON CPE matches (migration)</t>
+          <t>JSON CPE match objects (migration)</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1194,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>IOC value</t>
+          <t>Normalized IOC value</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1248,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>JSON result</t>
+          <t>JSON enrichment result</t>
         </is>
       </c>
     </row>
@@ -1246,10 +1268,14 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>6h TTL anchor</t>
+          <t>TTL anchor (6h reads)</t>
         </is>
       </c>
     </row>
@@ -1283,12 +1309,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>feed_cache</t>
+          <t>kev_deadlines</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>cache_key</t>
+          <t>product</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1296,26 +1322,22 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Cache key</t>
+          <t>KEV product name</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sync_state</t>
+          <t>kev_deadlines</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>short_description</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1323,26 +1345,22 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>PRIMARY KEY</t>
-        </is>
-      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>e.g. nvd_last_mod_end</t>
+          <t>CISA short text</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>epss_history</t>
+          <t>kev_deadlines</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>cve_id</t>
+          <t>required_action</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1350,53 +1368,45 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>PK part</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CVE ID</t>
+          <t>Remediation action</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>epss_history</t>
+          <t>kev_deadlines</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>score</t>
+          <t>due_date</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>REAL</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>NOT NULL</t>
-        </is>
-      </c>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>EPSS snapshot</t>
+          <t>Federal due date</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>epss_history</t>
+          <t>kev_deadlines</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>recorded_date</t>
+          <t>date_added</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1404,26 +1414,22 @@
           <t>TEXT</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>PK part</t>
-        </is>
-      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>KEV catalog add date</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>otx_cve_pulses</t>
+          <t>kev_deadlines</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>cve_id</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1433,24 +1439,24 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>PK part</t>
+          <t>DEFAULT datetime('now')</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CVE ID</t>
+          <t>Sync timestamp</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>otx_cve_pulses</t>
+          <t>api_usage</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>pulse_id</t>
+          <t>service</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1460,24 +1466,24 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>PK part</t>
+          <t>NOT NULL, PK part</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OTX pulse</t>
+          <t>Service slug e.g. nvd</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>correlation_infrastructure</t>
+          <t>api_usage</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>cve_id_a</t>
+          <t>date_utc</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1487,24 +1493,24 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>PK part</t>
+          <t>NOT NULL, PK part</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CVE A</t>
+          <t>YYYY-MM-DD</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>correlation_infrastructure</t>
+          <t>api_usage</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>cve_id_b</t>
+          <t>month_utc</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1514,51 +1520,51 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>PK part</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CVE B</t>
+          <t>YYYY-MM</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>correlation_actor</t>
+          <t>api_usage</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>cve_id</t>
+          <t>count</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>TEXT</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>PK part</t>
+          <t>DEFAULT 0</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CVE ID</t>
+          <t>Calls that day</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>correlation_actor</t>
+          <t>sync_state</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>actor_name</t>
+          <t>key</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1568,24 +1574,24 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>PK part</t>
+          <t>PRIMARY KEY</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Actor name</t>
+          <t>e.g. nvd_last_mod_end</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>correlation_temporal</t>
+          <t>sync_state</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>vendor</t>
+          <t>value</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1595,24 +1601,24 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
+          <t>NOT NULL</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Vendor slug</t>
+          <t>Watermark value</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>mitre_techniques</t>
+          <t>sync_state</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>technique_id</t>
+          <t>updated_at</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1622,19 +1628,15 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>PRIMARY KEY</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Txxxx</t>
-        </is>
-      </c>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>atlas_techniques</t>
+          <t>mitre_techniques</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1654,36 +1656,2029 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>AML.Txxxx</t>
+          <t>e.g. T1190</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>mitre_techniques</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Technique name</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>mitre_techniques</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>mitre_techniques</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>tactic</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Tactic name</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>mitre_techniques</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>attack.mitre.org URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>mitre_techniques</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>platforms</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>JSON platforms</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>mitre_techniques</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>detection</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Detection guidance</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>cve_technique_map</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>cve_id</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>cve_technique_map</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>technique_id</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>FK → mitre_techniques</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>atlas_techniques</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>technique_id</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>e.g. AML.T0051</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>atlas_techniques</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>atlas_techniques</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>atlas_techniques</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>tactic</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>atlas_techniques</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>tactic_id</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>atlas_techniques</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>atlas.mitre.org URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>atlas_case_studies</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>study_id</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>atlas_case_studies</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>atlas_case_studies</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>summary</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>atlas_case_studies</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>summary_full</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>atlas_case_studies</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>techniques</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>JSON technique IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>atlas_case_studies</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>atlas_case_studies</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>atlas_case_studies</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>study_type</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>atlas_case_studies</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>cve_ids</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>JSON CVE IDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>cve_atlas_map</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>cve_id</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>cve_atlas_map</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>technique_id</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>FK → atlas_techniques</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>epss_history</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>cve_id</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>epss_history</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>EPSS at snapshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>epss_history</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>recorded_date</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>cve_exploits</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY AUTOINCREMENT</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>cve_exploits</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>cve_id</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>cve_exploits</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>cve_exploits</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT 'poc'</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>cve_exploits</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>cve_exploits</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>cve_exploits</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>published_date</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>cve_exploits</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>fetched_at</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>feed_cache</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>cache_key</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>e.g. sploitus:CVE-...</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>feed_cache</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>JSON blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>feed_cache</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>cached_at</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>TTL checked at read</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>cve_change_history</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY AUTOINCREMENT</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>cve_change_history</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>cve_id</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>cve_change_history</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>field_name</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Tracked field</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>cve_change_history</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>old_value</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>cve_change_history</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>new_value</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>cve_change_history</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>detected_at</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>cve_id</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>pulse_id</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>pulse_name</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>created_date</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>adversary</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>malware_families</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ioc_count</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>tags</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>otx_cve_pulses</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>fetched_at</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>otx_pulse_iocs</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>pulse_id</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>otx_pulse_iocs</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ioc_type</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>NOT NULL DEFAULT '', PK part</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>otx_pulse_iocs</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>ioc_value</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>otx_pulse_iocs</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>otx_pulse_iocs</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>fetched_at</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>correlation_infrastructure</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>cve_id_a</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>correlation_infrastructure</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>cve_id_b</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>correlation_infrastructure</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>shared_ip_count</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>correlation_infrastructure</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>DEFAULT 'low'</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>correlation_infrastructure</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>detected_at</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>correlation_actor</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>cve_id</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>correlation_actor</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>actor_name</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>correlation_actor</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>actor_sectors</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>correlation_actor</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>user_sector_match</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>correlation_actor</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>DEFAULT 'low'</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>correlation_actor</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>detected_at</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>correlation_temporal</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>vendor</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>PRIMARY KEY</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>correlation_temporal</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>current_week_count</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>correlation_temporal</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>average_weekly_count</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>correlation_temporal</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>anomaly_score</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>DEFAULT 0</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>correlation_temporal</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>detected_at</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>DEFAULT datetime('now')</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
           <t>mitre_groups</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B115" t="inlineStr">
         <is>
           <t>group_id</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
         <is>
           <t>PRIMARY KEY</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Gxxxx</t>
-        </is>
-      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>e.g. G0016</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>mitre_groups</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>NOT NULL</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>mitre_groups</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>aliases</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>mitre_groups</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>mitre_groups</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>sectors</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>DEFAULT '[]'</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>JSON targeted sectors</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>mitre_groups</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>DEFAULT ''</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>group_technique_map</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>group_id</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>group_technique_map</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>technique_id</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>NOT NULL, PK part</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1974,14 +3969,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2029,12 +4024,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>50 req/30s with key</t>
+          <t>50/30s with key</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Retry/backoff</t>
+          <t>Retry/backoff; anonymous fallback</t>
         </is>
       </c>
     </row>
@@ -2046,7 +4041,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>cisa.gov/.../known_exploited_vulnerabilities.json</t>
+          <t>known_exploited_vulnerabilities.json</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -2069,7 +4064,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>epss.empiricalsecurity.com CSV</t>
+          <t>CSV gzip + api.first.org/data/v1/epss</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -2087,189 +4082,362 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>VirusTotal</t>
+          <t>MITRE STIX</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>virustotal.com/api/v3</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>VIRUSTOTAL_API_KEY</t>
-        </is>
-      </c>
+          <t>enterprise-attack.json + CTID CSV</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>500/day</t>
+          <t>Unlimited</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Empty fields</t>
+          <t>Job fails</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AbuseIPDB</t>
+          <t>ATLAS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>api.abuseipdb.com</t>
+          <t>GitHub raw YAML + case-studies API</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ABUSEIPDB_API_KEY</t>
+          <t>ATLAS_YAML_URL</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1000/day</t>
+          <t>Unlimited</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Skipped</t>
+          <t>Job fails</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GreyNoise</t>
+          <t>Sploitus</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>api.greynoise.io</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>GREYNOISE_API_KEY</t>
-        </is>
-      </c>
+          <t>sploitus.com search API</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>50/week</t>
+          <t>Unpublished</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>None/[]</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>OTX</t>
+          <t>GreyNoise</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>otx.alienvault.com/api/v1</t>
+          <t>api.greynoise.io/v3/community</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>OTX_API_KEY</t>
+          <t>GREYNOISE_API_KEY</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10k/month</t>
+          <t>50/week</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>Unknown classification</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Groq</t>
+          <t>VirusTotal</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>api.groq.com</t>
+          <t>virustotal.com/api/v3</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GROQ_API_KEY</t>
+          <t>VIRUSTOTAL_API_KEY</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Console quota</t>
+          <t>500/day</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Anthropic/template</t>
+          <t>Empty fields</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>AbuseIPDB</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>api.anthropic.com</t>
+          <t>api.abuseipdb.com/api/v2/check</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ANTHROPIC_API_KEY</t>
+          <t>ABUSEIPDB_API_KEY</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Console quota</t>
+          <t>1000/day</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Template</t>
+          <t>Skipped</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>OTX</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>otx.alienvault.com/api/v1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>OTX_API_KEY</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>10k/month</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OSV</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>api.osv.dev/v1/query</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CIRCL</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>cve.circl.lu/api/cve</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Unlimited</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No merge</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MalwareBazaar</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bazaar.abuse.ch/api</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ABUSECH_AUTH_KEY</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Fair use</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>URLhaus</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>urlhaus-api.abuse.ch</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ABUSECH_AUTH_KEY</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Fair use</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Groq</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>api.groq.com/openai/v1/chat/completions</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>GROQ_API_KEY</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Console quota</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Anthropic/template</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>api.anthropic.com/v1/messages</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Console quota</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Template</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>GitHub</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>api.github.com/search/code</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>GITHUB_TOKEN</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>60/hr anon</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>[]</t>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>60/hr without token</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>[] rules</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: AI/ML alerts, incidents feed performance, docs sync
- Wire ai_ml_alerts stat chip end-to-end (stats API, CVE filters, App)
- Add GET /api/case-studies/feed with parallel RSS + ATLAS load
- Client session cache for Incidents tab; remove dead AIThreats/riskScore
- Create Beta V1.2.md roadmap; update API_REFERENCE, SYSTEM_DESIGN,
  APPLICATION_EXECUTION_MAP, TECHNICAL_INVENTORY, README, xlsx generator
- Add backend tests for AI alerts and combined feed (75 tests passing)

Co-authored-by: Soldier0x0 <Soldier0x0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/TECHNICAL_INVENTORY.xlsx
+++ b/TECHNICAL_INVENTORY.xlsx
@@ -4664,12 +4664,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="57" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4765,19 +4765,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>API does not return atlas_techniques</t>
+          <t>has_ai_context + atlas_techniques on GET /api/cves/{id}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IOC lookup</t>
+          <t>AI/ML alerts stat</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4787,14 +4787,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>6h cache</t>
+          <t>GET /api/stats?frameworks= + feed filter</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Risk score v1.1b</t>
+          <t>Incidents combined feed</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -4804,14 +4804,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Client-side</t>
+          <t>GET /api/case-studies/feed parallel load</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Correlation</t>
+          <t>IOC lookup</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4828,7 +4828,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Detection tab</t>
+          <t>Risk score v1.1b</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4838,14 +4838,14 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sigma/Elastic</t>
+          <t>Client-side</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PDF + AI summary</t>
+          <t>Correlation</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4855,58 +4855,109 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Groq/Anthropic/template</t>
+          <t>6h cache</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>POST /api/investigation/summary</t>
+          <t>Detection tab</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Broken</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Undefined import main.py:1331</t>
+          <t>Sigma/Elastic</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>PDF + AI summary</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Not implemented</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>v1.1 by design</t>
+          <t>Groq/Anthropic/template</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Backups</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>6h timer, retention 100, auto-restore</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>POST /api/investigation/summary</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Legacy alias to generate_executive_summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Authentication</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Not implemented</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Planned v1.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Repository pattern</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Not implemented</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>v1.2</t>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Planned v1.2</t>
         </is>
       </c>
     </row>

</xml_diff>